<commit_message>
Update latest evolutions result
</commit_message>
<xml_diff>
--- a/latest/evolutions_raw_latest.xlsx
+++ b/latest/evolutions_raw_latest.xlsx
@@ -1088,12 +1088,12 @@
       </c>
       <c r="CX2" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 Details Submit by in 10 days Expiry in 17 days Coins Cost 35,000 Points Cost 250</t>
+          <t>Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 Details Submit by in 9 days Expiry in 16 days Coins Cost 35,000 Points Cost 250</t>
         </is>
       </c>
       <c r="CY2" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 Details Submit by in 10 days Expiry in 17 days Coins Cost 35,000 Points Cost 250</t>
+          <t>Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 Details Submit by in 9 days Expiry in 16 days Coins Cost 35,000 Points Cost 250</t>
         </is>
       </c>
       <c r="CZ2" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="DA2" t="inlineStr">
         <is>
-          <t>Maestro Unbound NEW 35,000 250 2 Unlock the true playmaking abilities of a player by adding all passing PlayStyles. Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 90.6 Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 92.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 UPGRADES 8 in 10 days in 17 days 25% 75%</t>
+          <t>Maestro Unbound NEW 35,000 250 2 Unlock the true playmaking abilities of a player by adding all passing PlayStyles. Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 90.6 Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 92.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 UPGRADES 8 in 9 days in 16 days 26% 74%</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="CX3" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 Details Submit by in 9 days Expiry in 16 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 Details Submit by in 8 days Expiry in 15 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY3" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 Details Submit by in 9 days Expiry in 16 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 Details Submit by in 8 days Expiry in 15 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ3" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="DA3" t="inlineStr">
         <is>
-          <t>Cat Like Reflexes Elevate your goalkeeper with elite-level reactions boosts designed to turn split-second moments into match-winning saves. Casillas 90 GK DIV 90 HAN 88 KIC 84 REF 93 SPD 59 POS 88 L 1 ★ 3 GK 83.1 Casillas 92 GK DIV 90 HAN 91 KIC 90 REF 94 SPD 69 POS 92 L 1 ★ 4 GK 87.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 UPGRADES +15 OVR 92 +15 POS 92 +1 WF +10 Acceleration 82 +10 Sprint Speed 82 +25 Reactions 93 +15 Diving 90 +15 Handling 91 +15 Kicking 90 +15 Reflexes 94 GK Goalkeeper ++ GK Ball Playing Keeper ++ GK Sweeper Keeper ++ 2 8 Show less in 9 days in 16 days 90% 10%</t>
+          <t>Cat Like Reflexes Elevate your goalkeeper with elite-level reactions boosts designed to turn split-second moments into match-winning saves. Casillas 90 GK DIV 90 HAN 88 KIC 84 REF 93 SPD 59 POS 88 L 1 ★ 3 GK 83.1 Casillas 92 GK DIV 90 HAN 91 KIC 90 REF 94 SPD 69 POS 92 L 1 ★ 4 GK 87.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 UPGRADES +15 OVR 92 +15 POS 92 +1 WF +10 Acceleration 82 +10 Sprint Speed 82 +25 Reactions 93 +15 Diving 90 +15 Handling 91 +15 Kicking 90 +15 Reflexes 94 GK Goalkeeper ++ GK Ball Playing Keeper ++ GK Sweeper Keeper ++ 2 8 Show less in 8 days in 15 days 90% 10%</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="CX4" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 Details Submit by in 8 days Expiry in 15 days Coins Cost 125,000 Points Cost 750</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 Details Submit by in 7 days Expiry in 14 days Coins Cost 125,000 Points Cost 750</t>
         </is>
       </c>
       <c r="CY4" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 Details Submit by in 8 days Expiry in 15 days Coins Cost 125,000 Points Cost 750</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 Details Submit by in 7 days Expiry in 14 days Coins Cost 125,000 Points Cost 750</t>
         </is>
       </c>
       <c r="CZ4" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="DA4" t="inlineStr">
         <is>
-          <t>Le Président 125,000 750 Transform your CB with the defensive excellence that made Laurent Blanc one of the greatest. Cool, composed, and unbeatable. Laporte 90 CB PAC 85 SHO 60 PAS 87 DRI 84 DEF 91 PHY 90 L 5 ★ 5 CB 79.3 Laporte 92 CB PAC 88 SHO 61 PAS 87 DRI 89 DEF 93 PHY 92 L 5 ★ 5 CB 91.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 UPGRADES +20 OVR 92 +3 WF 4 +30 Composure 92 +25 Aggression 90 +30 Short Pass 90 +30 Reactions 92 +30 Defensive Awareness 93 +30 Interceptions 92 +25 Stamina 90 +30 Heading Acc. 90 +20 Dribbling 87 +20 Sprint Speed 90 +25 Strength 91 +20 Balance 87 +25 Penalties 94 +30 Standing Tackle 94 +20 Acceleration 86 +20 Agility 88 +30 Long Pass 90 +25 Jumping 88 +30 Sliding Tackle 92 +30 Ball Control 92 3 7 in 8 days in 15 days 59% 41%</t>
+          <t>Le Président 125,000 750 Transform your CB with the defensive excellence that made Laurent Blanc one of the greatest. Cool, composed, and unbeatable. Laporte 90 CB PAC 85 SHO 60 PAS 87 DRI 84 DEF 91 PHY 90 L 5 ★ 5 CB 79.3 Laporte 92 CB PAC 88 SHO 61 PAS 87 DRI 89 DEF 93 PHY 92 L 5 ★ 5 CB 91.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 UPGRADES +20 OVR 92 +3 WF 4 +30 Composure 92 +25 Aggression 90 +30 Short Pass 90 +30 Reactions 92 +30 Defensive Awareness 93 +30 Interceptions 92 +25 Stamina 90 +30 Heading Acc. 90 +20 Dribbling 87 +20 Sprint Speed 90 +25 Strength 91 +20 Balance 87 +25 Penalties 94 +30 Standing Tackle 94 +20 Acceleration 86 +20 Agility 88 +30 Long Pass 90 +25 Jumping 88 +30 Sliding Tackle 92 +30 Ball Control 92 3 7 in 7 days in 14 days 59% 41%</t>
         </is>
       </c>
     </row>
@@ -1717,12 +1717,12 @@
       </c>
       <c r="CX5" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Details Submit by in 7 days Expiry in 14 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Details Submit by in 6 days Expiry in 13 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY5" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Details Submit by in 7 days Expiry in 14 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Details Submit by in 6 days Expiry in 13 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ5" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="DA5" t="inlineStr">
         <is>
-          <t>Lucky Number Seven 3 Hit your stride with Lucky Number Seven and give your eligible player boosts across key stats. Riise 88 LB PAC 88 SHO 83 PAS 86 DRI 85 DEF 86 PHY 88 LM L 4 ★ 4 LB 88.2 Riise 89 LB PAC 88 SHO 83 PAS 88 DRI 89 DEF 86 PHY 91 LM L 4 ★ 4 LB 89.5 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 UPGRADES +1 OVR +7 Shot Power 95 +7 Vision 92 +7 Crossing 93 +7 Balance 90 +7 Dribbling 93 +7 Jumping 92 +7 Strength 92 in 7 days in 14 days 26% 74%</t>
+          <t>Lucky Number Seven 3 Hit your stride with Lucky Number Seven and give your eligible player boosts across key stats. Riise 88 LB PAC 88 SHO 83 PAS 86 DRI 85 DEF 86 PHY 88 LM L 4 ★ 4 LB 88.2 Riise 89 LB PAC 88 SHO 83 PAS 88 DRI 89 DEF 86 PHY 91 LM L 4 ★ 4 LB 89.5 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 UPGRADES +1 OVR +7 Shot Power 95 +7 Vision 92 +7 Crossing 93 +7 Balance 90 +7 Dribbling 93 +7 Jumping 92 +7 Strength 92 in 6 days in 13 days 26% 74%</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="CX6" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 6 days Expiry in 13 days Coins Cost 35,000 Points Cost 200</t>
+          <t>Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 5 days Expiry in 12 days Coins Cost 35,000 Points Cost 200</t>
         </is>
       </c>
       <c r="CY6" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 6 days Expiry in 13 days Coins Cost 35,000 Points Cost 200</t>
+          <t>Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 5 days Expiry in 12 days Coins Cost 35,000 Points Cost 200</t>
         </is>
       </c>
       <c r="CZ6" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="DA6" t="inlineStr">
         <is>
-          <t>Fullback Takeover 35,000 200 Speed at the back. Power in every duel. A certain alpine player once ruled the center with unexpected power. Shift the role, break the line, and rediscover that unstoppable edge. Kimmich 89 RB PAC 81 SHO 74 PAS 89 DRI 85 DEF 85 PHY 80 CDM CM R 3 ★ 4 RB 81.0 Kimmich 90 RB PAC 91 SHO 74 PAS 89 DRI 85 DEF 90 PHY 88 CB CDM CM R 3 ★ 4 RB 89.7 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +15 OVR 90 +15 PAS 87 CB +2 WF 4 +20 Interceptions 91 +15 Strength 88 +20 Standing Tackle 90 +20 Defensive Awareness 91 +20 Stamina 92 +10 Composure 88 +10 Balance 86 +20 Acceleration 89 +15 Aggression 86 +20 Heading Acc. 83 +20 Sprint Speed 92 +10 Agility 88 +15 Jumping 88 +20 Sliding Tackle 93 +10 Reactions 88 3 7 Show less in 6 days in 13 days 22% 78%</t>
+          <t>Fullback Takeover 35,000 200 Speed at the back. Power in every duel. A certain alpine player once ruled the center with unexpected power. Shift the role, break the line, and rediscover that unstoppable edge. Kimmich 89 RB PAC 81 SHO 74 PAS 89 DRI 85 DEF 85 PHY 80 CDM CM R 3 ★ 4 RB 81.0 Kimmich 90 RB PAC 91 SHO 74 PAS 89 DRI 85 DEF 90 PHY 88 CB CDM CM R 3 ★ 4 RB 89.7 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +15 OVR 90 +15 PAS 87 CB +2 WF 4 +20 Interceptions 91 +15 Strength 88 +20 Standing Tackle 90 +20 Defensive Awareness 91 +20 Stamina 92 +10 Composure 88 +10 Balance 86 +20 Acceleration 89 +15 Aggression 86 +20 Heading Acc. 83 +20 Sprint Speed 92 +10 Agility 88 +15 Jumping 88 +20 Sliding Tackle 93 +10 Reactions 88 3 7 Show less in 5 days in 12 days 22% 78%</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="CX7" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 Details Submit by in 5 days Expiry in 12 days Coins Cost 75,000 Points Cost 400</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 Details Submit by in 4 days Expiry in 11 days Coins Cost 75,000 Points Cost 400</t>
         </is>
       </c>
       <c r="CY7" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 Details Submit by in 5 days Expiry in 12 days Coins Cost 75,000 Points Cost 400</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 Details Submit by in 4 days Expiry in 11 days Coins Cost 75,000 Points Cost 400</t>
         </is>
       </c>
       <c r="CZ7" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="DA7" t="inlineStr">
         <is>
-          <t>Gear 5 75,000 400 Hit the gear and let loose with +5 boosts across key stats. Bounce past rivals, stretch the game, and chase victory with a grin. Davies 89 LB PAC 95 SHO 80 PAS 84 DRI 87 DEF 82 PHY 84 LM L 4 ★ 3 LB 87.9 Davies 91 LB PAC 95 SHO 83 PAS 86 DRI 91 DEF 86 PHY 87 LM L 5 ★ 5 LB 91.2 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 UPGRADES +5 OVR 91 +4 SM +4 WF +5 Sliding Tackle 90 +5 Vision 91 +5 Sprint Speed 89 +5 Crossing 86 +5 Long Pass 90 +5 Interceptions 88 +5 Volleys 86 +5 Composure 87 +5 Heading Acc. 85 +5 Curve 90 +5 Agility 92 +5 Positioning 91 +5 Standing Tackle 86 +5 Finishing 89 +5 Reactions 90 +5 Balance 92 +5 Strength 86 +5 Short Pass 90 +5 Jumping 90 +5 Long Shots 87 +5 Stamina 90 +5 Defensive Awareness 86 +5 Ball Control 91 +5 Dribbling 92 +5 Aggression 86 +5 Shot Power 88 +5 Acceleration 89 in 5 days in 12 days 8% 92%</t>
+          <t>Gear 5 75,000 400 Hit the gear and let loose with +5 boosts across key stats. Bounce past rivals, stretch the game, and chase victory with a grin. Davies 89 LB PAC 95 SHO 80 PAS 84 DRI 87 DEF 82 PHY 84 LM L 4 ★ 3 LB 87.9 Davies 91 LB PAC 95 SHO 83 PAS 86 DRI 91 DEF 86 PHY 87 LM L 5 ★ 5 LB 91.2 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 UPGRADES +5 OVR 91 +4 SM +4 WF +5 Sliding Tackle 90 +5 Vision 91 +5 Sprint Speed 89 +5 Crossing 86 +5 Long Pass 90 +5 Interceptions 88 +5 Volleys 86 +5 Composure 87 +5 Heading Acc. 85 +5 Curve 90 +5 Agility 92 +5 Positioning 91 +5 Standing Tackle 86 +5 Finishing 89 +5 Reactions 90 +5 Balance 92 +5 Strength 86 +5 Short Pass 90 +5 Jumping 90 +5 Long Shots 87 +5 Stamina 90 +5 Defensive Awareness 86 +5 Ball Control 91 +5 Dribbling 92 +5 Aggression 86 +5 Shot Power 88 +5 Acceleration 89 in 4 days in 11 days 8% 92%</t>
         </is>
       </c>
     </row>
@@ -2458,12 +2458,12 @@
       </c>
       <c r="CX8" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 Details Submit by in 4 days Expiry in 11 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 10 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY8" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 Details Submit by in 4 days Expiry in 11 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 10 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ8" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="DA8" t="inlineStr">
         <is>
-          <t>Steel Guard 3 Cold as steel and impossible to break, dominates every duel, reads the game perfectly, and shuts down attacks before they even become a threat. Zima 74 CB PAC 76 SHO 38 PAS 54 DRI 62 DEF 75 PHY 75 R 2 ★ 4 CB 65.6 Zima 74 CB PAC 77 SHO 38 PAS 55 DRI 62 DEF 77 PHY 75 R 2 ★ 4 CB 75.9 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 UPGRADES +2 Sliding Tackle 78 +2 Short Pass 78 +2 Defensive Awareness 80 +2 Interceptions 80 +1 Jumping 75 +1 Sprint Speed 80 +2 Standing Tackle 80 +1 Acceleration 80 +1 Strength 78 +2 Vision 72 +1 Aggression 75 +1 Stamina 78 +2 Heading Acc. 76 2 8 in 4 days in 11 days 7% 93%</t>
+          <t>Steel Guard 3 Cold as steel and impossible to break, dominates every duel, reads the game perfectly, and shuts down attacks before they even become a threat. Zima 74 CB PAC 76 SHO 38 PAS 54 DRI 62 DEF 75 PHY 75 R 2 ★ 4 CB 65.6 Zima 74 CB PAC 77 SHO 38 PAS 55 DRI 62 DEF 77 PHY 75 R 2 ★ 4 CB 75.9 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 UPGRADES +2 Sliding Tackle 78 +2 Short Pass 78 +2 Defensive Awareness 80 +2 Interceptions 80 +1 Jumping 75 +1 Sprint Speed 80 +2 Standing Tackle 80 +1 Acceleration 80 +1 Strength 78 +2 Vision 72 +1 Aggression 75 +1 Stamina 78 +2 Heading Acc. 76 2 8 in 3 days in 10 days 7% 93%</t>
         </is>
       </c>
     </row>
@@ -2723,12 +2723,12 @@
       </c>
       <c r="CX9" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 10 days Coins Cost 50,000 Points Cost 300</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 2 days Expiry in 9 days Coins Cost 50,000 Points Cost 300</t>
         </is>
       </c>
       <c r="CY9" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 10 days Coins Cost 50,000 Points Cost 300</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 Details Submit by in 2 days Expiry in 9 days Coins Cost 50,000 Points Cost 300</t>
         </is>
       </c>
       <c r="CZ9" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="DA9" t="inlineStr">
         <is>
-          <t>Lightning Wingback 50,000 300 Lightning-fast wingback to dominate the flank. Explosive pace, relentless overlaps, and pinpoint delivery. A constant threat in attack while tracking back with power and precision. Savona 83 RB PAC 84 SHO 57 PAS 75 DRI 76 DEF 83 PHY 83 LB RM R 2 ★ 3 RB 80.1 Savona 91 RB PAC 93 SHO 64 PAS 81 DRI 90 DEF 90 PHY 92 LB RM R 2 ★ 5 RB 94.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +30 OVR 91 +4 WF +35 Standing Tackle 87 +25 Aggression 92 +30 Sprint Speed 93 +50 Positioning 90 +30 Crossing 94 +30 Composure 89 +30 Acceleration 93 +30 Dribbling 89 +35 Interceptions 92 +30 Short Pass 92 +50 Long Pass 93 +35 Defensive Awareness 90 +30 Balance 90 +30 Agility 90 +20 Stamina 94 +50 Shot Power 94 +35 Sliding Tackle 95 +20 Jumping 90 +35 Heading Acc. 92 +30 Reactions 93 +30 Ball Control 90 +25 Strength 91 3 7 in 3 days in 10 days 91% 9%</t>
+          <t>Lightning Wingback 50,000 300 Lightning-fast wingback to dominate the flank. Explosive pace, relentless overlaps, and pinpoint delivery. A constant threat in attack while tracking back with power and precision. Savona 83 RB PAC 84 SHO 57 PAS 75 DRI 76 DEF 83 PHY 83 LB RM R 2 ★ 3 RB 80.1 Savona 91 RB PAC 93 SHO 64 PAS 81 DRI 90 DEF 90 PHY 92 LB RM R 2 ★ 5 RB 94.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +30 OVR 91 +4 WF +35 Standing Tackle 87 +25 Aggression 92 +30 Sprint Speed 93 +50 Positioning 90 +30 Crossing 94 +30 Composure 89 +30 Acceleration 93 +30 Dribbling 89 +35 Interceptions 92 +30 Short Pass 92 +50 Long Pass 93 +35 Defensive Awareness 90 +30 Balance 90 +30 Agility 90 +20 Stamina 94 +50 Shot Power 94 +35 Sliding Tackle 95 +20 Jumping 90 +35 Heading Acc. 92 +30 Reactions 93 +30 Ball Control 90 +25 Strength 91 3 7 in 2 days in 9 days 91% 9%</t>
         </is>
       </c>
     </row>
@@ -2902,12 +2902,12 @@
       </c>
       <c r="CX10" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 Details Submit by in 2 days Expiry in 9 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 Details Submit by in 1 day Expiry in 8 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY10" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 Details Submit by in 2 days Expiry in 9 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 Details Submit by in 1 day Expiry in 8 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ10" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="DA10" t="inlineStr">
         <is>
-          <t>Curve Your Enthusiasm 5 Bend the game to your will and create moments of magic by transforming a player into a ball-bending specialist. Bobb 88 RW PAC 93 SHO 87 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 88.2 Bobb 88 RW PAC 93 SHO 90 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 89.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 UPGRADES +3 Positioning 90 +5 Finishing 92 +5 Long Shots 92 +3 Shot Power 90 +8 Curve 95 8 in 2 days in 9 days 31% 69%</t>
+          <t>Curve Your Enthusiasm 5 Bend the game to your will and create moments of magic by transforming a player into a ball-bending specialist. Bobb 88 RW PAC 93 SHO 87 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 88.2 Bobb 88 RW PAC 93 SHO 90 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 89.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 UPGRADES +3 Positioning 90 +5 Finishing 92 +5 Long Shots 92 +3 Shot Power 90 +8 Curve 95 8 in 1 day in 8 days 31% 69%</t>
         </is>
       </c>
     </row>
@@ -3145,12 +3145,12 @@
       </c>
       <c r="CX11" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 Details Submit by in 13 hours Expiry in 8 days Coins Cost 100,000 Points Cost 500</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 Details Submit by in 11 hours Expiry in 7 days Coins Cost 100,000 Points Cost 500</t>
         </is>
       </c>
       <c r="CY11" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 Details Submit by in 13 hours Expiry in 8 days Coins Cost 100,000 Points Cost 500</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 Details Submit by in 11 hours Expiry in 7 days Coins Cost 100,000 Points Cost 500</t>
         </is>
       </c>
       <c r="CZ11" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="DA11" t="inlineStr">
         <is>
-          <t>Cut In, Say Less 100,000 500 Elevate your favourite qualified player with enhanced pace, dribbling, shooting, and passing, allowing them to cut inside, get past defenders, and deliver in decisive moments! Debinha 89 RW PAC 87 SHO 82 PAS 87 DRI 92 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 86.5 Debinha 92 RW PAC 92 SHO 90 PAS 92 DRI 93 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 93.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 UPGRADES +17 OVR 92 +4 SM 5 +17 Acceleration 93 +17 Sprint Speed 91 +17 Vision 93 +17 Crossing 90 +17 Fk Accuracy 89 +17 Short Pass 92 +17 Long Pass 91 +17 Agility 94 +17 Balance 92 +17 Reactions 91 +17 Ball Control 91 +17 Dribbling 92 +17 Composure 91 +17 Curve 94 +17 Finishing 92 +17 Shot Power 91 +17 Long Shots 90 +17 Volleys 86 3 7 in 13 hours in 8 days 64% 36%</t>
+          <t>Cut In, Say Less 100,000 500 Elevate your favourite qualified player with enhanced pace, dribbling, shooting, and passing, allowing them to cut inside, get past defenders, and deliver in decisive moments! Debinha 89 RW PAC 87 SHO 82 PAS 87 DRI 92 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 86.5 Debinha 92 RW PAC 92 SHO 90 PAS 92 DRI 93 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 93.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 UPGRADES +17 OVR 92 +4 SM 5 +17 Acceleration 93 +17 Sprint Speed 91 +17 Vision 93 +17 Crossing 90 +17 Fk Accuracy 89 +17 Short Pass 92 +17 Long Pass 91 +17 Agility 94 +17 Balance 92 +17 Reactions 91 +17 Ball Control 91 +17 Dribbling 92 +17 Composure 91 +17 Curve 94 +17 Finishing 92 +17 Shot Power 91 +17 Long Shots 90 +17 Volleys 86 3 7 in 11 hours in 7 days 64% 36%</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="DA17" t="inlineStr">
         <is>
-          <t>Rapid+ Unlocked by completing the Assist in 10 task in the Ligue 1 TOTS Exhibition objective Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 84.0 Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 85.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS+ 2 UPGRADES 3 in 9 days in 9 days 92% 8%</t>
+          <t>Rapid+ Unlocked by completing the Assist in 10 task in the Ligue 1 TOTS Exhibition objective Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 84.0 Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 85.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS+ 2 UPGRADES 3 in 9 days in 9 days 91% 9%</t>
         </is>
       </c>
     </row>
@@ -7082,12 +7082,12 @@
       </c>
       <c r="CX34" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 3 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 Details Submit by in 2 days Expiry in 2 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY34" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 Details Submit by in 3 days Expiry in 3 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 Details Submit by in 2 days Expiry in 2 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ34" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="DA34" t="inlineStr">
         <is>
-          <t>Welsh Wonder Strike [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lukaku 85 CAM PAC 84 SHO 86 PAS 80 DRI 81 DEF 42 PHY 85 ST L 4 ★ 4 ST 80.4 Lukaku 89 CAM PAC 92 SHO 90 PAS 86 DRI 89 DEF 42 PHY 85 ST L 4 ★ 4 ST 90.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 UPGRADES +15 OVR 89 +25 Acceleration 90 +20 Shot Power 90 +10 Vision 87 +25 Composure 88 +25 Sprint Speed 93 +20 Long Shots 90 +10 Long Pass 87 +25 Dribbling 90 +20 Positioning 89 +20 Volleys 93 +15 Short Pass 88 +25 Ball Control 89 +30 Jumping 92 +20 Finishing 90 +10 Crossing 86 +15 Curve 89 +25 Reactions 90 +20 Heading Acc. 87 +20 Penalties 87 +15 Fk Accuracy 88 +25 Agility 88 +25 Balance 87 2 8 TRAINING TIME 31 minutes in 3 days in 3 days 18% 82%</t>
+          <t>Welsh Wonder Strike [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lukaku 85 CAM PAC 84 SHO 86 PAS 80 DRI 81 DEF 42 PHY 85 ST L 4 ★ 4 ST 80.4 Lukaku 89 CAM PAC 92 SHO 90 PAS 86 DRI 89 DEF 42 PHY 85 ST L 4 ★ 4 ST 90.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 UPGRADES +15 OVR 89 +25 Acceleration 90 +20 Shot Power 90 +10 Vision 87 +25 Composure 88 +25 Sprint Speed 93 +20 Long Shots 90 +10 Long Pass 87 +25 Dribbling 90 +20 Positioning 89 +20 Volleys 93 +15 Short Pass 88 +25 Ball Control 89 +30 Jumping 92 +20 Finishing 90 +10 Crossing 86 +15 Curve 89 +25 Reactions 90 +20 Heading Acc. 87 +20 Penalties 87 +15 Fk Accuracy 88 +25 Agility 88 +25 Balance 87 2 8 TRAINING TIME 31 minutes in 2 days in 2 days 18% 82%</t>
         </is>
       </c>
     </row>
@@ -7345,12 +7345,12 @@
       </c>
       <c r="CX35" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 Details Submit by in 3 days Expiry in 3 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 Details Submit by in 2 days Expiry in 2 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CY35" t="inlineStr">
         <is>
-          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 Details Submit by in 3 days Expiry in 3 days Coins Cost Free Points Cost Free</t>
+          <t>Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 Details Submit by in 2 days Expiry in 2 days Coins Cost Free Points Cost Free</t>
         </is>
       </c>
       <c r="CZ35" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="DA35" t="inlineStr">
         <is>
-          <t>Il Capitano [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lawrence 70 CB PAC 60 SHO 26 PAS 49 DRI 46 DEF 70 PHY 73 R 2 ★ 2 CB 62.3 Lawrence 91 CB PAC 88 SHO 26 PAS 68 DRI 72 DEF 93 PHY 90 R 2 ★ 2 CB 92.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 UPGRADES +30 OVR 91 +30 Acceleration 87 +30 Short Pass 90 +30 Heading Acc. 92 +30 Defensive Awareness 95 +30 Sprint Speed 88 +30 Vision 70 +30 Agility 73 +30 Balance 80 +30 Long Pass 85 +30 Ball Control 75 +30 Dribbling 75 +30 Reactions 95 +30 Composure 91 +30 Interceptions 93 +30 Standing Tackle 92 +30 Sliding Tackle 92 +30 Stamina 90 +30 Strength 92 +30 Jumping 90 +30 Aggression 85 CB Defender ++ CB Stopper ++ CB Wideback ++ 2 8 in 3 days in 3 days 19% 81%</t>
+          <t>Il Capitano [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lawrence 70 CB PAC 60 SHO 26 PAS 49 DRI 46 DEF 70 PHY 73 R 2 ★ 2 CB 62.3 Lawrence 91 CB PAC 88 SHO 26 PAS 68 DRI 72 DEF 93 PHY 90 R 2 ★ 2 CB 92.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 UPGRADES +30 OVR 91 +30 Acceleration 87 +30 Short Pass 90 +30 Heading Acc. 92 +30 Defensive Awareness 95 +30 Sprint Speed 88 +30 Vision 70 +30 Agility 73 +30 Balance 80 +30 Long Pass 85 +30 Ball Control 75 +30 Dribbling 75 +30 Reactions 95 +30 Composure 91 +30 Interceptions 93 +30 Standing Tackle 92 +30 Sliding Tackle 92 +30 Stamina 90 +30 Strength 92 +30 Jumping 90 +30 Aggression 85 CB Defender ++ CB Stopper ++ CB Wideback ++ 2 8 in 2 days in 2 days 19% 81%</t>
         </is>
       </c>
     </row>
@@ -65689,7 +65689,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Maestro Unbound NEW 35,000 250 2 Unlock the true playmaking abilities of a player by adding all passing PlayStyles. Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 90.6 Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 92.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 UPGRADES 8 in 10 days in 17 days 25% 75%</t>
+          <t>Maestro Unbound NEW 35,000 250 2 Unlock the true playmaking abilities of a player by adding all passing PlayStyles. Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 90.6 Pelé 96 CAM PAC 94 SHO 96 PAS 92 DRI 95 DEF 60 PHY 75 ST R 5 ★ 4 CAM 92.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max PS 7 Max PS+ 2 UPGRADES 8 in 9 days in 16 days 26% 74%</t>
         </is>
       </c>
     </row>
@@ -65716,7 +65716,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cat Like Reflexes Elevate your goalkeeper with elite-level reactions boosts designed to turn split-second moments into match-winning saves. Casillas 90 GK DIV 90 HAN 88 KIC 84 REF 93 SPD 59 POS 88 L 1 ★ 3 GK 83.1 Casillas 92 GK DIV 90 HAN 91 KIC 90 REF 94 SPD 69 POS 92 L 1 ★ 4 GK 87.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 UPGRADES +15 OVR 92 +15 POS 92 +1 WF +10 Acceleration 82 +10 Sprint Speed 82 +25 Reactions 93 +15 Diving 90 +15 Handling 91 +15 Kicking 90 +15 Reflexes 94 GK Goalkeeper ++ GK Ball Playing Keeper ++ GK Sweeper Keeper ++ 2 8 Show less in 9 days in 16 days 90% 10%</t>
+          <t>Cat Like Reflexes Elevate your goalkeeper with elite-level reactions boosts designed to turn split-second moments into match-winning saves. Casillas 90 GK DIV 90 HAN 88 KIC 84 REF 93 SPD 59 POS 88 L 1 ★ 3 GK 83.1 Casillas 92 GK DIV 90 HAN 91 KIC 90 REF 94 SPD 69 POS 92 L 1 ★ 4 GK 87.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position GK Max PS 10 Max PS+ 2 UPGRADES +15 OVR 92 +15 POS 92 +1 WF +10 Acceleration 82 +10 Sprint Speed 82 +25 Reactions 93 +15 Diving 90 +15 Handling 91 +15 Kicking 90 +15 Reflexes 94 GK Goalkeeper ++ GK Ball Playing Keeper ++ GK Sweeper Keeper ++ 2 8 Show less in 8 days in 15 days 90% 10%</t>
         </is>
       </c>
     </row>
@@ -65743,7 +65743,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Le Président 125,000 750 Transform your CB with the defensive excellence that made Laurent Blanc one of the greatest. Cool, composed, and unbeatable. Laporte 90 CB PAC 85 SHO 60 PAS 87 DRI 84 DEF 91 PHY 90 L 5 ★ 5 CB 79.3 Laporte 92 CB PAC 88 SHO 61 PAS 87 DRI 89 DEF 93 PHY 92 L 5 ★ 5 CB 91.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 UPGRADES +20 OVR 92 +3 WF 4 +30 Composure 92 +25 Aggression 90 +30 Short Pass 90 +30 Reactions 92 +30 Defensive Awareness 93 +30 Interceptions 92 +25 Stamina 90 +30 Heading Acc. 90 +20 Dribbling 87 +20 Sprint Speed 90 +25 Strength 91 +20 Balance 87 +25 Penalties 94 +30 Standing Tackle 94 +20 Acceleration 86 +20 Agility 88 +30 Long Pass 90 +25 Jumping 88 +30 Sliding Tackle 92 +30 Ball Control 92 3 7 in 8 days in 15 days 59% 41%</t>
+          <t>Le Président 125,000 750 Transform your CB with the defensive excellence that made Laurent Blanc one of the greatest. Cool, composed, and unbeatable. Laporte 90 CB PAC 85 SHO 60 PAS 87 DRI 84 DEF 91 PHY 90 L 5 ★ 5 CB 79.3 Laporte 92 CB PAC 88 SHO 61 PAS 87 DRI 89 DEF 93 PHY 92 L 5 ★ 5 CB 91.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position CB Max PS 10 Max PS+ 2 Heading Accuracy Max. 94 UPGRADES +20 OVR 92 +3 WF 4 +30 Composure 92 +25 Aggression 90 +30 Short Pass 90 +30 Reactions 92 +30 Defensive Awareness 93 +30 Interceptions 92 +25 Stamina 90 +30 Heading Acc. 90 +20 Dribbling 87 +20 Sprint Speed 90 +25 Strength 91 +20 Balance 87 +25 Penalties 94 +30 Standing Tackle 94 +20 Acceleration 86 +20 Agility 88 +30 Long Pass 90 +25 Jumping 88 +30 Sliding Tackle 92 +30 Ball Control 92 3 7 in 7 days in 14 days 59% 41%</t>
         </is>
       </c>
     </row>
@@ -65770,7 +65770,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lucky Number Seven 3 Hit your stride with Lucky Number Seven and give your eligible player boosts across key stats. Riise 88 LB PAC 88 SHO 83 PAS 86 DRI 85 DEF 86 PHY 88 LM L 4 ★ 4 LB 88.2 Riise 89 LB PAC 88 SHO 83 PAS 88 DRI 89 DEF 86 PHY 91 LM L 4 ★ 4 LB 89.5 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 UPGRADES +1 OVR +7 Shot Power 95 +7 Vision 92 +7 Crossing 93 +7 Balance 90 +7 Dribbling 93 +7 Jumping 92 +7 Strength 92 in 7 days in 14 days 26% 74%</t>
+          <t>Lucky Number Seven 3 Hit your stride with Lucky Number Seven and give your eligible player boosts across key stats. Riise 88 LB PAC 88 SHO 83 PAS 86 DRI 85 DEF 86 PHY 88 LM L 4 ★ 4 LB 88.2 Riise 89 LB PAC 88 SHO 83 PAS 88 DRI 89 DEF 86 PHY 91 LM L 4 ★ 4 LB 89.5 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 UPGRADES +1 OVR +7 Shot Power 95 +7 Vision 92 +7 Crossing 93 +7 Balance 90 +7 Dribbling 93 +7 Jumping 92 +7 Strength 92 in 6 days in 13 days 26% 74%</t>
         </is>
       </c>
     </row>
@@ -65797,7 +65797,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fullback Takeover 35,000 200 Speed at the back. Power in every duel. A certain alpine player once ruled the center with unexpected power. Shift the role, break the line, and rediscover that unstoppable edge. Kimmich 89 RB PAC 81 SHO 74 PAS 89 DRI 85 DEF 85 PHY 80 CDM CM R 3 ★ 4 RB 81.0 Kimmich 90 RB PAC 91 SHO 74 PAS 89 DRI 85 DEF 90 PHY 88 CB CDM CM R 3 ★ 4 RB 89.7 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +15 OVR 90 +15 PAS 87 CB +2 WF 4 +20 Interceptions 91 +15 Strength 88 +20 Standing Tackle 90 +20 Defensive Awareness 91 +20 Stamina 92 +10 Composure 88 +10 Balance 86 +20 Acceleration 89 +15 Aggression 86 +20 Heading Acc. 83 +20 Sprint Speed 92 +10 Agility 88 +15 Jumping 88 +20 Sliding Tackle 93 +10 Reactions 88 3 7 Show less in 6 days in 13 days 22% 78%</t>
+          <t>Fullback Takeover 35,000 200 Speed at the back. Power in every duel. A certain alpine player once ruled the center with unexpected power. Shift the role, break the line, and rediscover that unstoppable edge. Kimmich 89 RB PAC 81 SHO 74 PAS 89 DRI 85 DEF 85 PHY 80 CDM CM R 3 ★ 4 RB 81.0 Kimmich 90 RB PAC 91 SHO 74 PAS 89 DRI 85 DEF 90 PHY 88 CB CDM CM R 3 ★ 4 RB 89.7 REQUIREMENTS Excluded Rarity World Tour Silver Stars Max Pos. 3 Overall Max. 89 Position RB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +15 OVR 90 +15 PAS 87 CB +2 WF 4 +20 Interceptions 91 +15 Strength 88 +20 Standing Tackle 90 +20 Defensive Awareness 91 +20 Stamina 92 +10 Composure 88 +10 Balance 86 +20 Acceleration 89 +15 Aggression 86 +20 Heading Acc. 83 +20 Sprint Speed 92 +10 Agility 88 +15 Jumping 88 +20 Sliding Tackle 93 +10 Reactions 88 3 7 Show less in 5 days in 12 days 22% 78%</t>
         </is>
       </c>
     </row>
@@ -65824,7 +65824,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Gear 5 75,000 400 Hit the gear and let loose with +5 boosts across key stats. Bounce past rivals, stretch the game, and chase victory with a grin. Davies 89 LB PAC 95 SHO 80 PAS 84 DRI 87 DEF 82 PHY 84 LM L 4 ★ 3 LB 87.9 Davies 91 LB PAC 95 SHO 83 PAS 86 DRI 91 DEF 86 PHY 87 LM L 5 ★ 5 LB 91.2 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 UPGRADES +5 OVR 91 +4 SM +4 WF +5 Sliding Tackle 90 +5 Vision 91 +5 Sprint Speed 89 +5 Crossing 86 +5 Long Pass 90 +5 Interceptions 88 +5 Volleys 86 +5 Composure 87 +5 Heading Acc. 85 +5 Curve 90 +5 Agility 92 +5 Positioning 91 +5 Standing Tackle 86 +5 Finishing 89 +5 Reactions 90 +5 Balance 92 +5 Strength 86 +5 Short Pass 90 +5 Jumping 90 +5 Long Shots 87 +5 Stamina 90 +5 Defensive Awareness 86 +5 Ball Control 91 +5 Dribbling 92 +5 Aggression 86 +5 Shot Power 88 +5 Acceleration 89 in 5 days in 12 days 8% 92%</t>
+          <t>Gear 5 75,000 400 Hit the gear and let loose with +5 boosts across key stats. Bounce past rivals, stretch the game, and chase victory with a grin. Davies 89 LB PAC 95 SHO 80 PAS 84 DRI 87 DEF 82 PHY 84 LM L 4 ★ 3 LB 87.9 Davies 91 LB PAC 95 SHO 83 PAS 86 DRI 91 DEF 86 PHY 87 LM L 5 ★ 5 LB 91.2 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS 10 Max PS+ 2 UPGRADES +5 OVR 91 +4 SM +4 WF +5 Sliding Tackle 90 +5 Vision 91 +5 Sprint Speed 89 +5 Crossing 86 +5 Long Pass 90 +5 Interceptions 88 +5 Volleys 86 +5 Composure 87 +5 Heading Acc. 85 +5 Curve 90 +5 Agility 92 +5 Positioning 91 +5 Standing Tackle 86 +5 Finishing 89 +5 Reactions 90 +5 Balance 92 +5 Strength 86 +5 Short Pass 90 +5 Jumping 90 +5 Long Shots 87 +5 Stamina 90 +5 Defensive Awareness 86 +5 Ball Control 91 +5 Dribbling 92 +5 Aggression 86 +5 Shot Power 88 +5 Acceleration 89 in 4 days in 11 days 8% 92%</t>
         </is>
       </c>
     </row>
@@ -65851,7 +65851,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Steel Guard 3 Cold as steel and impossible to break, dominates every duel, reads the game perfectly, and shuts down attacks before they even become a threat. Zima 74 CB PAC 76 SHO 38 PAS 54 DRI 62 DEF 75 PHY 75 R 2 ★ 4 CB 65.6 Zima 74 CB PAC 77 SHO 38 PAS 55 DRI 62 DEF 77 PHY 75 R 2 ★ 4 CB 75.9 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 UPGRADES +2 Sliding Tackle 78 +2 Short Pass 78 +2 Defensive Awareness 80 +2 Interceptions 80 +1 Jumping 75 +1 Sprint Speed 80 +2 Standing Tackle 80 +1 Acceleration 80 +1 Strength 78 +2 Vision 72 +1 Aggression 75 +1 Stamina 78 +2 Heading Acc. 76 2 8 in 4 days in 11 days 7% 93%</t>
+          <t>Steel Guard 3 Cold as steel and impossible to break, dominates every duel, reads the game perfectly, and shuts down attacks before they even become a threat. Zima 74 CB PAC 76 SHO 38 PAS 54 DRI 62 DEF 75 PHY 75 R 2 ★ 4 CB 65.6 Zima 74 CB PAC 77 SHO 38 PAS 55 DRI 62 DEF 77 PHY 75 R 2 ★ 4 CB 75.9 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 74 Max PS 10 Max PS+ 2 UPGRADES +2 Sliding Tackle 78 +2 Short Pass 78 +2 Defensive Awareness 80 +2 Interceptions 80 +1 Jumping 75 +1 Sprint Speed 80 +2 Standing Tackle 80 +1 Acceleration 80 +1 Strength 78 +2 Vision 72 +1 Aggression 75 +1 Stamina 78 +2 Heading Acc. 76 2 8 in 3 days in 10 days 7% 93%</t>
         </is>
       </c>
     </row>
@@ -65878,7 +65878,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Lightning Wingback 50,000 300 Lightning-fast wingback to dominate the flank. Explosive pace, relentless overlaps, and pinpoint delivery. A constant threat in attack while tracking back with power and precision. Savona 83 RB PAC 84 SHO 57 PAS 75 DRI 76 DEF 83 PHY 83 LB RM R 2 ★ 3 RB 80.1 Savona 91 RB PAC 93 SHO 64 PAS 81 DRI 90 DEF 90 PHY 92 LB RM R 2 ★ 5 RB 94.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +30 OVR 91 +4 WF +35 Standing Tackle 87 +25 Aggression 92 +30 Sprint Speed 93 +50 Positioning 90 +30 Crossing 94 +30 Composure 89 +30 Acceleration 93 +30 Dribbling 89 +35 Interceptions 92 +30 Short Pass 92 +50 Long Pass 93 +35 Defensive Awareness 90 +30 Balance 90 +30 Agility 90 +20 Stamina 94 +50 Shot Power 94 +35 Sliding Tackle 95 +20 Jumping 90 +35 Heading Acc. 92 +30 Reactions 93 +30 Ball Control 90 +25 Strength 91 3 7 in 3 days in 10 days 91% 9%</t>
+          <t>Lightning Wingback 50,000 300 Lightning-fast wingback to dominate the flank. Explosive pace, relentless overlaps, and pinpoint delivery. A constant threat in attack while tracking back with power and precision. Savona 83 RB PAC 84 SHO 57 PAS 75 DRI 76 DEF 83 PHY 83 LB RM R 2 ★ 3 RB 80.1 Savona 91 RB PAC 93 SHO 64 PAS 81 DRI 90 DEF 90 PHY 92 LB RM R 2 ★ 5 RB 94.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position LB Excluded Position CB Max PS 10 Max PS+ 2 UPGRADES +30 OVR 91 +4 WF +35 Standing Tackle 87 +25 Aggression 92 +30 Sprint Speed 93 +50 Positioning 90 +30 Crossing 94 +30 Composure 89 +30 Acceleration 93 +30 Dribbling 89 +35 Interceptions 92 +30 Short Pass 92 +50 Long Pass 93 +35 Defensive Awareness 90 +30 Balance 90 +30 Agility 90 +20 Stamina 94 +50 Shot Power 94 +35 Sliding Tackle 95 +20 Jumping 90 +35 Heading Acc. 92 +30 Reactions 93 +30 Ball Control 90 +25 Strength 91 3 7 in 2 days in 9 days 91% 9%</t>
         </is>
       </c>
     </row>
@@ -65905,7 +65905,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Curve Your Enthusiasm 5 Bend the game to your will and create moments of magic by transforming a player into a ball-bending specialist. Bobb 88 RW PAC 93 SHO 87 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 88.2 Bobb 88 RW PAC 93 SHO 90 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 89.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 UPGRADES +3 Positioning 90 +5 Finishing 92 +5 Long Shots 92 +3 Shot Power 90 +8 Curve 95 8 in 2 days in 9 days 31% 69%</t>
+          <t>Curve Your Enthusiasm 5 Bend the game to your will and create moments of magic by transforming a player into a ball-bending specialist. Bobb 88 RW PAC 93 SHO 87 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 88.2 Bobb 88 RW PAC 93 SHO 90 PAS 88 DRI 93 DEF 48 PHY 69 RM LW L 5 ★ 4 RM 89.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 88 Max PS 10 UPGRADES +3 Positioning 90 +5 Finishing 92 +5 Long Shots 92 +3 Shot Power 90 +8 Curve 95 8 in 1 day in 8 days 31% 69%</t>
         </is>
       </c>
     </row>
@@ -65932,7 +65932,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cut In, Say Less 100,000 500 Elevate your favourite qualified player with enhanced pace, dribbling, shooting, and passing, allowing them to cut inside, get past defenders, and deliver in decisive moments! Debinha 89 RW PAC 87 SHO 82 PAS 87 DRI 92 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 86.5 Debinha 92 RW PAC 92 SHO 90 PAS 92 DRI 93 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 93.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 UPGRADES +17 OVR 92 +4 SM 5 +17 Acceleration 93 +17 Sprint Speed 91 +17 Vision 93 +17 Crossing 90 +17 Fk Accuracy 89 +17 Short Pass 92 +17 Long Pass 91 +17 Agility 94 +17 Balance 92 +17 Reactions 91 +17 Ball Control 91 +17 Dribbling 92 +17 Composure 91 +17 Curve 94 +17 Finishing 92 +17 Shot Power 91 +17 Long Shots 90 +17 Volleys 86 3 7 in 13 hours in 8 days 64% 36%</t>
+          <t>Cut In, Say Less 100,000 500 Elevate your favourite qualified player with enhanced pace, dribbling, shooting, and passing, allowing them to cut inside, get past defenders, and deliver in decisive moments! Debinha 89 RW PAC 87 SHO 82 PAS 87 DRI 92 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 86.5 Debinha 92 RW PAC 92 SHO 90 PAS 92 DRI 93 DEF 48 PHY 78 RM CM CAM R 5 ★ 5 RM 93.3 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 90 Position RM, RW Max PS 10 Max PS+ 2 UPGRADES +17 OVR 92 +4 SM 5 +17 Acceleration 93 +17 Sprint Speed 91 +17 Vision 93 +17 Crossing 90 +17 Fk Accuracy 89 +17 Short Pass 92 +17 Long Pass 91 +17 Agility 94 +17 Balance 92 +17 Reactions 91 +17 Ball Control 91 +17 Dribbling 92 +17 Composure 91 +17 Curve 94 +17 Finishing 92 +17 Shot Power 91 +17 Long Shots 90 +17 Volleys 86 3 7 in 11 hours in 7 days 64% 36%</t>
         </is>
       </c>
     </row>
@@ -66094,7 +66094,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Rapid+ Unlocked by completing the Assist in 10 task in the Ligue 1 TOTS Exhibition objective Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 84.0 Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 85.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS+ 2 UPGRADES 3 in 9 days in 9 days 92% 8%</t>
+          <t>Rapid+ Unlocked by completing the Assist in 10 task in the Ligue 1 TOTS Exhibition objective Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 84.0 Yılmaz 89 LM PAC 97 SHO 86 PAS 85 DRI 89 DEF 81 PHY 95 RM LW R 5 ★ 5 LM 85.8 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Max PS+ 2 UPGRADES 3 in 9 days in 9 days 91% 9%</t>
         </is>
       </c>
     </row>
@@ -66553,7 +66553,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Welsh Wonder Strike [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lukaku 85 CAM PAC 84 SHO 86 PAS 80 DRI 81 DEF 42 PHY 85 ST L 4 ★ 4 ST 80.4 Lukaku 89 CAM PAC 92 SHO 90 PAS 86 DRI 89 DEF 42 PHY 85 ST L 4 ★ 4 ST 90.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 UPGRADES +15 OVR 89 +25 Acceleration 90 +20 Shot Power 90 +10 Vision 87 +25 Composure 88 +25 Sprint Speed 93 +20 Long Shots 90 +10 Long Pass 87 +25 Dribbling 90 +20 Positioning 89 +20 Volleys 93 +15 Short Pass 88 +25 Ball Control 89 +30 Jumping 92 +20 Finishing 90 +10 Crossing 86 +15 Curve 89 +25 Reactions 90 +20 Heading Acc. 87 +20 Penalties 87 +15 Fk Accuracy 88 +25 Agility 88 +25 Balance 87 2 8 TRAINING TIME 31 minutes in 3 days in 3 days 18% 82%</t>
+          <t>Welsh Wonder Strike [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lukaku 85 CAM PAC 84 SHO 86 PAS 80 DRI 81 DEF 42 PHY 85 ST L 4 ★ 4 ST 80.4 Lukaku 89 CAM PAC 92 SHO 90 PAS 86 DRI 89 DEF 42 PHY 85 ST L 4 ★ 4 ST 90.1 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 87 Max PS 10 Max PS+ 2 UPGRADES +15 OVR 89 +25 Acceleration 90 +20 Shot Power 90 +10 Vision 87 +25 Composure 88 +25 Sprint Speed 93 +20 Long Shots 90 +10 Long Pass 87 +25 Dribbling 90 +20 Positioning 89 +20 Volleys 93 +15 Short Pass 88 +25 Ball Control 89 +30 Jumping 92 +20 Finishing 90 +10 Crossing 86 +15 Curve 89 +25 Reactions 90 +20 Heading Acc. 87 +20 Penalties 87 +15 Fk Accuracy 88 +25 Agility 88 +25 Balance 87 2 8 TRAINING TIME 31 minutes in 2 days in 2 days 18% 82%</t>
         </is>
       </c>
     </row>
@@ -66580,7 +66580,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Il Capitano [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lawrence 70 CB PAC 60 SHO 26 PAS 49 DRI 46 DEF 70 PHY 73 R 2 ★ 2 CB 62.3 Lawrence 91 CB PAC 88 SHO 26 PAS 68 DRI 72 DEF 93 PHY 90 R 2 ★ 2 CB 92.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 UPGRADES +30 OVR 91 +30 Acceleration 87 +30 Short Pass 90 +30 Heading Acc. 92 +30 Defensive Awareness 95 +30 Sprint Speed 88 +30 Vision 70 +30 Agility 73 +30 Balance 80 +30 Long Pass 85 +30 Ball Control 75 +30 Dribbling 75 +30 Reactions 95 +30 Composure 91 +30 Interceptions 93 +30 Standing Tackle 92 +30 Sliding Tackle 92 +30 Stamina 90 +30 Strength 92 +30 Jumping 90 +30 Aggression 85 CB Defender ++ CB Stopper ++ CB Wideback ++ 2 8 in 3 days in 3 days 19% 81%</t>
+          <t>Il Capitano [Store] Unlocked by purchasing the Captains' Armband EVO pack. Lawrence 70 CB PAC 60 SHO 26 PAS 49 DRI 46 DEF 70 PHY 73 R 2 ★ 2 CB 62.3 Lawrence 91 CB PAC 88 SHO 26 PAS 68 DRI 72 DEF 93 PHY 90 R 2 ★ 2 CB 92.6 REQUIREMENTS Excluded Rarity World Tour Silver Stars Overall Max. 89 Position CB Excluded Position CM Max PS 10 Max PS+ 2 Pace Max. 90 UPGRADES +30 OVR 91 +30 Acceleration 87 +30 Short Pass 90 +30 Heading Acc. 92 +30 Defensive Awareness 95 +30 Sprint Speed 88 +30 Vision 70 +30 Agility 73 +30 Balance 80 +30 Long Pass 85 +30 Ball Control 75 +30 Dribbling 75 +30 Reactions 95 +30 Composure 91 +30 Interceptions 93 +30 Standing Tackle 92 +30 Sliding Tackle 92 +30 Stamina 90 +30 Strength 92 +30 Jumping 90 +30 Aggression 85 CB Defender ++ CB Stopper ++ CB Wideback ++ 2 8 in 2 days in 2 days 19% 81%</t>
         </is>
       </c>
     </row>
@@ -68136,7 +68136,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-11T04:11:09</t>
+          <t>2026-05-11T06:00:54</t>
         </is>
       </c>
     </row>

</xml_diff>